<commit_message>
Updated testing documentation for phase 2 and 4
</commit_message>
<xml_diff>
--- a/BankCoreSolution/BankCore.TestDocs/TestCases/TestCases - Excecuted.xlsx
+++ b/BankCoreSolution/BankCore.TestDocs/TestCases/TestCases - Excecuted.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jaydee Venter\Software Testing Simulation Project (WIL)\BankCoreSolution\BankCore.TestDocs\TestCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F629C01-6C2B-420B-BED9-D2C016C19620}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE28799-655D-446A-A4F0-F4E7E7C9626C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="824" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="824" firstSheet="1" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Account Management Test Cases" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,10 @@
     <sheet name="Reporting Engine Test Cases" sheetId="6" r:id="rId5"/>
     <sheet name="Authentication Test Cases" sheetId="7" r:id="rId6"/>
     <sheet name="Validation Library Test Cases" sheetId="8" r:id="rId7"/>
+    <sheet name="Decision Table" sheetId="9" r:id="rId8"/>
+    <sheet name="State Transition Table" sheetId="10" r:id="rId9"/>
+    <sheet name="Error Guessing Table" sheetId="12" r:id="rId10"/>
+    <sheet name="Non-Functional Test Cases" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1963" uniqueCount="758">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2257" uniqueCount="966">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -2684,12 +2688,640 @@
   <si>
     <t>Verify validation service rejects operations when session owner lacks required permissions.</t>
   </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Rule 1: 
+Is Account Active?</t>
+  </si>
+  <si>
+    <t>Rule 2:
+Does Account Have Sufficient Funds?</t>
+  </si>
+  <si>
+    <t>Rule 3:
+Under Daily Limit?</t>
+  </si>
+  <si>
+    <t>Expected Outcome</t>
+  </si>
+  <si>
+    <t>Expected Error Message If Not True</t>
+  </si>
+  <si>
+    <t>BEMS-DT-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRUE </t>
+  </si>
+  <si>
+    <t>Approve</t>
+  </si>
+  <si>
+    <t>None - All rules are true</t>
+  </si>
+  <si>
+    <t>BEMS-DT-02</t>
+  </si>
+  <si>
+    <t>Reject</t>
+  </si>
+  <si>
+    <t>Withdrawals can only be made from Active accounts.</t>
+  </si>
+  <si>
+    <t>BEMS-DT-03</t>
+  </si>
+  <si>
+    <t>Insufficient funds.</t>
+  </si>
+  <si>
+    <t>BEMS-DT-04</t>
+  </si>
+  <si>
+    <t>Daily withdrawal limit of R50000,00 would be exceeded.</t>
+  </si>
+  <si>
+    <t>BEMS-DT-05</t>
+  </si>
+  <si>
+    <t>BEMS-DT-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALSE </t>
+  </si>
+  <si>
+    <t>BEMS-DT-07</t>
+  </si>
+  <si>
+    <t>BEMS-DT-08</t>
+  </si>
+  <si>
+    <t>NF-PERF</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Threshold</t>
+  </si>
+  <si>
+    <t>Measured time</t>
+  </si>
+  <si>
+    <t>Recommendation</t>
+  </si>
+  <si>
+    <t>TC-BEMS-PERF-001</t>
+  </si>
+  <si>
+    <t>How long it takes for the program to run</t>
+  </si>
+  <si>
+    <t>The program should launch quickly, within ~5 seconds within clicking the login button</t>
+  </si>
+  <si>
+    <t>~2 seconds to launch the program</t>
+  </si>
+  <si>
+    <t>TC-BEMS-PERF-002</t>
+  </si>
+  <si>
+    <t>The time it takes to log into the system</t>
+  </si>
+  <si>
+    <t>The program should login within 0.5 seconds of clicking the login button</t>
+  </si>
+  <si>
+    <t>0.5 seconds to log into the program</t>
+  </si>
+  <si>
+    <t>TC-BEMS-PERF-003</t>
+  </si>
+  <si>
+    <t>How long it takes to generate a account transaction history with 200+ transactions</t>
+  </si>
+  <si>
+    <t>15 to 20 seconds for a large report</t>
+  </si>
+  <si>
+    <t>Report generated in 12 seconds</t>
+  </si>
+  <si>
+    <t>TC-BEMS-PERF-004</t>
+  </si>
+  <si>
+    <t>How long transactions take when multiple tellers are performing transactions concurrently</t>
+  </si>
+  <si>
+    <t>Regular transactions should take around 2 seconds to process</t>
+  </si>
+  <si>
+    <t>Transactions process within 1.5 seconds with multiple transactions being performed at the same time</t>
+  </si>
+  <si>
+    <t>TC-BEMS-PERF-005</t>
+  </si>
+  <si>
+    <t>Testing how long the system takes to run a system audit log of 1 year</t>
+  </si>
+  <si>
+    <t>System should take around 10 to 15 minutes to generate the detailed system audit log</t>
+  </si>
+  <si>
+    <t>The system took 14 minutes to generate the complete systemlog</t>
+  </si>
+  <si>
+    <t>TC-BEMS-PERF-006</t>
+  </si>
+  <si>
+    <t>Testing to see how well the program performs after 24 hours of continuous operations being performed on it</t>
+  </si>
+  <si>
+    <t>The program should see a very slight degradation in performance, and should take around 1 to 2 seconds to process transactions</t>
+  </si>
+  <si>
+    <t>Program took 1 second to process transactions</t>
+  </si>
+  <si>
+    <t>NF-ROB</t>
+  </si>
+  <si>
+    <t>Input used</t>
+  </si>
+  <si>
+    <t>Expected handling</t>
+  </si>
+  <si>
+    <t>Actual result</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ROBUST-001</t>
+  </si>
+  <si>
+    <t>Numbers in a string only field</t>
+  </si>
+  <si>
+    <t>The program should display an error message to the user stating that only alphabetical characters are allowed</t>
+  </si>
+  <si>
+    <t>The program successfully rejects the input, and displays a message stating Alphabetic characters only</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ROBUST-002</t>
+  </si>
+  <si>
+    <t>Entering alphabetical characters into a numerical only field</t>
+  </si>
+  <si>
+    <t>The system should reject the input, and display an error message static invalid input</t>
+  </si>
+  <si>
+    <t>The program displays an error message stating that only numerical fields are allowed</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ROBUST-003</t>
+  </si>
+  <si>
+    <t>Attempting to transfer the maximum possible amount to transfer without the program crashing</t>
+  </si>
+  <si>
+    <t>The program should not crash, and instead should display an error message to the user stating the max amount they are allowed to enter</t>
+  </si>
+  <si>
+    <t>The program does not crash when the invalid amount is entered</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ROBUST-004</t>
+  </si>
+  <si>
+    <t>Entering a ID number that does not meet the correct length or format</t>
+  </si>
+  <si>
+    <t>The program should handle this input error without the system crashing</t>
+  </si>
+  <si>
+    <t>The system displays an error message stating that the ID number entered is not valid.</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ROBUST-005</t>
+  </si>
+  <si>
+    <t>Entering a password below the minimum allowed length</t>
+  </si>
+  <si>
+    <t>The system should reject the password, and display an error message stating that the password does not meet length requirements</t>
+  </si>
+  <si>
+    <t>The program displays an error message stating that the password does not meet the length requirements</t>
+  </si>
+  <si>
+    <t>NF-SEC</t>
+  </si>
+  <si>
+    <t>Test performed</t>
+  </si>
+  <si>
+    <t>Expected behavior</t>
+  </si>
+  <si>
+    <t>Actual behavior</t>
+  </si>
+  <si>
+    <t>Risk rating (if failed)</t>
+  </si>
+  <si>
+    <t>TC-BEMS-SEC-001</t>
+  </si>
+  <si>
+    <t>Logging in with invalid credentials</t>
+  </si>
+  <si>
+    <t>The program should not allow the user to login</t>
+  </si>
+  <si>
+    <t>TC-BEMS-SEC-002</t>
+  </si>
+  <si>
+    <t>Attempting to access admin features as a standard user</t>
+  </si>
+  <si>
+    <t>The program should not allow the standard user to access administrator features</t>
+  </si>
+  <si>
+    <t>The program does not allow the standard user to access admin features</t>
+  </si>
+  <si>
+    <t>TC-BEMS-SEC-003</t>
+  </si>
+  <si>
+    <t>Session tokens expire upon logout</t>
+  </si>
+  <si>
+    <t>The program should expire the user session token upon logout</t>
+  </si>
+  <si>
+    <t>Then token is set to expire</t>
+  </si>
+  <si>
+    <t>TC-BEMS-SEC-004</t>
+  </si>
+  <si>
+    <t>SQL string injection prevention</t>
+  </si>
+  <si>
+    <t>The program should reject all SQL injection strings</t>
+  </si>
+  <si>
+    <t>The program rejects SQL injection strings</t>
+  </si>
+  <si>
+    <t>TC-BEMS-SEC-005</t>
+  </si>
+  <si>
+    <t>Strong password requirements</t>
+  </si>
+  <si>
+    <t>Program should have strong password requirements, and not allow past passwords to be used</t>
+  </si>
+  <si>
+    <t>The program has strong password requirements</t>
+  </si>
+  <si>
+    <t>TC-BEMS-SEC-006</t>
+  </si>
+  <si>
+    <t>Password hashing</t>
+  </si>
+  <si>
+    <t>Passwords should be hashed, and not displayed as plain text</t>
+  </si>
+  <si>
+    <t>All passwords are hashed</t>
+  </si>
+  <si>
+    <t>Account State Transition</t>
+  </si>
+  <si>
+    <t>Current State</t>
+  </si>
+  <si>
+    <t>Transition Trigger</t>
+  </si>
+  <si>
+    <t>Expected State</t>
+  </si>
+  <si>
+    <t>Actual State</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-001</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>Account is activated</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-002</t>
+  </si>
+  <si>
+    <t>Account is set to Dormant</t>
+  </si>
+  <si>
+    <t>Dormant</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-003</t>
+  </si>
+  <si>
+    <t>Customer diposits money</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-004</t>
+  </si>
+  <si>
+    <t>Customer requests account closure</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-005</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-006</t>
+  </si>
+  <si>
+    <t>Customer depositis money</t>
+  </si>
+  <si>
+    <t>Error message</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-007</t>
+  </si>
+  <si>
+    <t>Pending account</t>
+  </si>
+  <si>
+    <t>customer attemps deposit</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-008</t>
+  </si>
+  <si>
+    <t>Closed Account</t>
+  </si>
+  <si>
+    <t>Attempt to activate</t>
+  </si>
+  <si>
+    <t>TC-BEMS-ACCSTATE-009</t>
+  </si>
+  <si>
+    <t>Active Account</t>
+  </si>
+  <si>
+    <t>Loan Process State Transitions</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-001</t>
+  </si>
+  <si>
+    <t>Admin Approves</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-002</t>
+  </si>
+  <si>
+    <t>Does not meet requirements</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-003</t>
+  </si>
+  <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Customer miss a payment</t>
+  </si>
+  <si>
+    <t>Arrears</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-004</t>
+  </si>
+  <si>
+    <t>Customer makes a payment</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-005</t>
+  </si>
+  <si>
+    <t>Customer pays off the loan</t>
+  </si>
+  <si>
+    <t>Settled</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-006</t>
+  </si>
+  <si>
+    <t>Customer attempts to close account</t>
+  </si>
+  <si>
+    <t>Error message thrown</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-007</t>
+  </si>
+  <si>
+    <t>Customer attempts to increase loan amount</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-008</t>
+  </si>
+  <si>
+    <t>Customer attempts to use loan</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-009</t>
+  </si>
+  <si>
+    <t>Attempt to approve loan</t>
+  </si>
+  <si>
+    <t>Remains dormant</t>
+  </si>
+  <si>
+    <t>Rejected</t>
+  </si>
+  <si>
+    <t>Settled (if exact amount is paid)
+Arrears (if over payment is made)</t>
+  </si>
+  <si>
+    <t>TC-BEMS-LOANSTATE-010</t>
+  </si>
+  <si>
+    <t>Customer starts using loan</t>
+  </si>
+  <si>
+    <t>Common Error Made</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>User leaves required fields empty</t>
+  </si>
+  <si>
+    <t>User leaves a mandatory field like ID open or blank</t>
+  </si>
+  <si>
+    <t>The program displays an error message</t>
+  </si>
+  <si>
+    <t>Teller attempts to perform admin actionq</t>
+  </si>
+  <si>
+    <t>A teller attempts to create an account</t>
+  </si>
+  <si>
+    <t>The program displays an error message stating that the teller does not have the correct permissions</t>
+  </si>
+  <si>
+    <t>Creating a audit reports with dates in the future</t>
+  </si>
+  <si>
+    <t>Generating a audit report, but the dates are in the future</t>
+  </si>
+  <si>
+    <t>The program must display an error message stating that the dates have not yet passed</t>
+  </si>
+  <si>
+    <t>Withdrawing an amount above the allowed daily limit</t>
+  </si>
+  <si>
+    <t>Attempt to withdraw a amount that exceeds daily allowed limit</t>
+  </si>
+  <si>
+    <t>The program rejects the withdrawal</t>
+  </si>
+  <si>
+    <t>Tranferring to an inactive account</t>
+  </si>
+  <si>
+    <t>Attemting to make a transfer bit the destination account is not active</t>
+  </si>
+  <si>
+    <t>The program should display an error message stating that the destination account is not active</t>
+  </si>
+  <si>
+    <t>Withdrawing money from an account with insufficient funds</t>
+  </si>
+  <si>
+    <t>A withdraw attempt is made from an account with invalid funds</t>
+  </si>
+  <si>
+    <t>The program should display an error message stating that the account does not have enough funds</t>
+  </si>
+  <si>
+    <t>Entering an invalid data type into a field</t>
+  </si>
+  <si>
+    <t>Attempting to enter a string in the user ID field</t>
+  </si>
+  <si>
+    <t>The program should display an error message stating that the field input may only be numerical</t>
+  </si>
+  <si>
+    <t>Changing a password that does not meet complexity requirements</t>
+  </si>
+  <si>
+    <t>Attempting to change user password that is not strong enough</t>
+  </si>
+  <si>
+    <t>The program displays an error message stating that the password does not meet minimum complexity requirements</t>
+  </si>
+  <si>
+    <t>Submitting a reversal on the same transaction ID twice</t>
+  </si>
+  <si>
+    <t>Attempting to make a reversal on the same transaction ID twice</t>
+  </si>
+  <si>
+    <t>The program should display an error message stating that the transaction has already been reversed</t>
+  </si>
+  <si>
+    <t>Overpaying when settling a loan</t>
+  </si>
+  <si>
+    <t>The user makes an overpayment when settling a loan</t>
+  </si>
+  <si>
+    <t>The program should only take the settlement amount, and If there is any extra, the account should be credited</t>
+  </si>
+  <si>
+    <t>Withdrawaling the exact account balance on a current account</t>
+  </si>
+  <si>
+    <t>The user withdrawals the exact amount of the account balance</t>
+  </si>
+  <si>
+    <t>The program should not allow the transaction to happen</t>
+  </si>
+  <si>
+    <t>Making a transfer, but omitting the reference</t>
+  </si>
+  <si>
+    <t>A transfer is performed, but the reference/description is left blank</t>
+  </si>
+  <si>
+    <t>The program should not allow the tranfer to happen</t>
+  </si>
+  <si>
+    <t>Program displays an invalid input error</t>
+  </si>
+  <si>
+    <t>Program displays a permissions required message</t>
+  </si>
+  <si>
+    <t>Program incorrectly generates the report</t>
+  </si>
+  <si>
+    <t>Program rejects the withdraw</t>
+  </si>
+  <si>
+    <t>Program displays a error message stating that transfers can only be made to active accounts</t>
+  </si>
+  <si>
+    <t>Program displays an insufficient funds message</t>
+  </si>
+  <si>
+    <t>Program displays a password does not meet requirements error</t>
+  </si>
+  <si>
+    <t>Program displays error message: "Transaction has already been revered" message</t>
+  </si>
+  <si>
+    <t>Program incorrectly sets account into arrears</t>
+  </si>
+  <si>
+    <t>Program allows the exact amount to be withdrawn</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2715,16 +3347,38 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor theme="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -2732,11 +3386,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2757,17 +3448,397 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="92">
+  <dxfs count="144">
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="medium">
+          <color theme="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="medium">
+          <color theme="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="1"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="1"/>
+        </left>
+        <right style="thin">
+          <color theme="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -3056,147 +4127,246 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}" name="Table1" displayName="Table1" ref="A1:L26" totalsRowShown="0" dataDxfId="78">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}" name="Table1" displayName="Table1" ref="A1:L26" totalsRowShown="0" dataDxfId="130">
   <autoFilter ref="A1:L26" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{A91B6F41-4D2A-41F1-9826-979068F814A6}" name="Test Case ID" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{60D40DF6-B6BE-4F37-BACF-DBB67B68904C}" name="Test Suite" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{18667E7B-6DD3-452C-B6AD-71956CB63156}" name="Test Title" dataDxfId="75"/>
-    <tableColumn id="4" xr3:uid="{CAEC85EE-ADE2-4B1C-84B2-FED1E5057C53}" name="Preconditions" dataDxfId="74"/>
-    <tableColumn id="5" xr3:uid="{214FB217-B0EA-40D2-867E-56EB85668737}" name="Test Steps" dataDxfId="73"/>
-    <tableColumn id="6" xr3:uid="{394C4348-5EC9-454A-A752-CFE1E6794DFF}" name="Expected Result" dataDxfId="72"/>
-    <tableColumn id="7" xr3:uid="{1111BF3B-968D-4F77-962C-F5DE55E5F624}" name="Actual Result" dataDxfId="71"/>
-    <tableColumn id="8" xr3:uid="{BEFA7A31-5C09-4A32-B5D9-D7A10D06A1FB}" name="Pass/Fail" dataDxfId="70"/>
-    <tableColumn id="9" xr3:uid="{E7BB23C6-DE72-4013-80F0-5BA84E649C34}" name="Defect Reference" dataDxfId="69"/>
-    <tableColumn id="10" xr3:uid="{552808F4-DE21-43E0-BDFB-EA530745C6CA}" name="Priority" dataDxfId="68"/>
-    <tableColumn id="11" xr3:uid="{BB463A97-7CA4-4890-8550-DA1CDB28BEB5}" name="Test Type" dataDxfId="67"/>
-    <tableColumn id="12" xr3:uid="{17C7B85D-3A36-4F1A-B5D6-79967EA4529A}" name="Technique Used" dataDxfId="66"/>
+    <tableColumn id="1" xr3:uid="{A91B6F41-4D2A-41F1-9826-979068F814A6}" name="Test Case ID" dataDxfId="129"/>
+    <tableColumn id="2" xr3:uid="{60D40DF6-B6BE-4F37-BACF-DBB67B68904C}" name="Test Suite" dataDxfId="128"/>
+    <tableColumn id="3" xr3:uid="{18667E7B-6DD3-452C-B6AD-71956CB63156}" name="Test Title" dataDxfId="127"/>
+    <tableColumn id="4" xr3:uid="{CAEC85EE-ADE2-4B1C-84B2-FED1E5057C53}" name="Preconditions" dataDxfId="126"/>
+    <tableColumn id="5" xr3:uid="{214FB217-B0EA-40D2-867E-56EB85668737}" name="Test Steps" dataDxfId="125"/>
+    <tableColumn id="6" xr3:uid="{394C4348-5EC9-454A-A752-CFE1E6794DFF}" name="Expected Result" dataDxfId="124"/>
+    <tableColumn id="7" xr3:uid="{1111BF3B-968D-4F77-962C-F5DE55E5F624}" name="Actual Result" dataDxfId="123"/>
+    <tableColumn id="8" xr3:uid="{BEFA7A31-5C09-4A32-B5D9-D7A10D06A1FB}" name="Pass/Fail" dataDxfId="122"/>
+    <tableColumn id="9" xr3:uid="{E7BB23C6-DE72-4013-80F0-5BA84E649C34}" name="Defect Reference" dataDxfId="121"/>
+    <tableColumn id="10" xr3:uid="{552808F4-DE21-43E0-BDFB-EA530745C6CA}" name="Priority" dataDxfId="120"/>
+    <tableColumn id="11" xr3:uid="{BB463A97-7CA4-4890-8550-DA1CDB28BEB5}" name="Test Type" dataDxfId="119"/>
+    <tableColumn id="12" xr3:uid="{17C7B85D-3A36-4F1A-B5D6-79967EA4529A}" name="Technique Used" dataDxfId="118"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="19" xr:uid="{91E99773-8F1E-4AF3-8320-B2ABE5864630}" name="Table14" displayName="Table14" ref="A13:E23" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" headerRowBorderDxfId="12" tableBorderDxfId="13">
+  <autoFilter ref="A13:E23" xr:uid="{91E99773-8F1E-4AF3-8320-B2ABE5864630}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{6500F65A-7EE6-4BCE-8F14-561E1B309636}" name="Test Case ID" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{41A7A2F2-EEBC-4072-832A-6EBB1B3D5201}" name="Current State" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{9508FF32-BD38-4300-A9E8-D0A4819FFF3D}" name="Transition Trigger" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{D330C616-4923-4FE0-9F21-DB8D7D9264B0}" name="Expected State" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{2AFDE5DC-1243-4913-AAE7-D14B9EDAAEF6}" name="Actual State" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="20" xr:uid="{80C75059-DE7C-4319-9A96-0F3CB16AF5CE}" name="Table15" displayName="Table15" ref="A1:D13" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:D13" xr:uid="{80C75059-DE7C-4319-9A96-0F3CB16AF5CE}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{56FB8F1E-4556-4A8B-B9C5-36CC34DA2362}" name="Common Error Made" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{FE753A40-9CE9-4867-9196-D262FAB76EB2}" name="Scenario" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{32F73C21-D565-4E7E-887C-03495779E768}" name="Expected Result" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{F6ADE743-9F8F-43B3-BA2A-123C903C8D0A}" name="Actual Result" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="15" xr:uid="{F91334A9-BC56-4DCD-8176-C33F6FC95701}" name="Table9" displayName="Table9" ref="A2:F8" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
+  <autoFilter ref="A2:F8" xr:uid="{F91334A9-BC56-4DCD-8176-C33F6FC95701}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{8DAB2AB4-90D2-4952-9994-536C668071B2}" name="Test Case ID" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{043BBB1D-BAD4-47E1-931B-21A93F4E8374}" name="Title" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{F97AD5B3-E7B6-4D5E-8BCD-5C492EF6CE3C}" name="Threshold" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{68E28220-845D-4A3C-8D52-FA88A8926362}" name="Measured time" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{0784602B-79A5-4C74-BE27-2B158379F276}" name="Pass/Fail" dataDxfId="38"/>
+    <tableColumn id="6" xr3:uid="{19B0D059-3BF9-4F23-AB6A-5E0C61C789CE}" name="Recommendation" dataDxfId="37"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="16" xr:uid="{60D9FCDC-C524-4E2C-9336-0E718EAE498E}" name="Table10" displayName="Table10" ref="A10:E15" totalsRowShown="0" headerRowDxfId="36" dataDxfId="35">
+  <autoFilter ref="A10:E15" xr:uid="{60D9FCDC-C524-4E2C-9336-0E718EAE498E}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{1B6F8C7E-5B2B-4E1E-B487-5CC9C078CB39}" name="Test Case ID" dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{8F0B372F-DF7D-4B87-AA0F-8683DB32F606}" name="Input used" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{6E17C7D1-08AB-465A-A746-DB6A3DE7CD73}" name="Expected handling" dataDxfId="32"/>
+    <tableColumn id="4" xr3:uid="{17FDD823-8440-4537-B236-E5E01504FB3D}" name="Actual result" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{468160FE-B2C6-455F-849F-AB0CC3BAC863}" name="Pass/Fail" dataDxfId="30"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{223A3868-3614-4152-8C7A-E85428E2FE56}" name="Table11" displayName="Table11" ref="A17:E23" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
+  <autoFilter ref="A17:E23" xr:uid="{223A3868-3614-4152-8C7A-E85428E2FE56}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{A8E0E866-CEB5-43E0-87F8-2A83ACAE039A}" name="Test Case ID" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{90DE930F-8B5E-4D8A-AA56-F69517DC8839}" name="Test performed" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{159A18B1-EF2A-4CF7-BA1D-87C43E39AA2F}" name="Expected behavior" dataDxfId="25"/>
+    <tableColumn id="4" xr3:uid="{5013CB7C-19DA-407F-9349-95C75172EBB5}" name="Actual behavior" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{6DFEF342-2228-4853-8470-26EA4150A053}" name="Risk rating (if failed)" dataDxfId="23"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{63B090D9-E720-47BB-9BC0-E7551EBCB5F4}" name="Table13" displayName="Table13" ref="A1:L35" totalsRowShown="0" dataDxfId="65">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{63B090D9-E720-47BB-9BC0-E7551EBCB5F4}" name="Table13" displayName="Table13" ref="A1:L35" totalsRowShown="0" dataDxfId="117">
   <autoFilter ref="A1:L35" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{2744E4B1-F4AF-4C38-A165-A36AFDC6ED20}" name="Test Case ID" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{025A828A-E3BB-46BB-9738-33A224653725}" name="Test Suite" dataDxfId="63"/>
-    <tableColumn id="3" xr3:uid="{63419378-8000-4158-90E8-6D8BFCDA2241}" name="Test Title" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{485947B2-61B2-4E7A-9F45-DEE2A6A31241}" name="Preconditions" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{694A91C3-2EF7-4662-BA6E-D1E59F3B94D5}" name="Test Steps" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{61B98F31-1685-42B6-BF1B-14C77B125CFB}" name="Expected Result" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{C5850C5A-CF04-45AE-AFF2-FF9A3159C7A6}" name="Actual Result" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{880E8ECB-3308-49AD-B50B-5CCE1EF7E617}" name="Pass/Fail" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{4F749DFF-645B-47DB-9AAC-12B65CE23CB3}" name="Defect Reference" dataDxfId="56"/>
-    <tableColumn id="10" xr3:uid="{A573EAAC-61E8-4701-AA89-F5788D455FC0}" name="Priority" dataDxfId="55"/>
-    <tableColumn id="11" xr3:uid="{8507D1F9-0769-438C-86B4-E44A8C17EF24}" name="Test Type" dataDxfId="54"/>
-    <tableColumn id="12" xr3:uid="{ADF76C2E-E815-4CC9-B9BC-DE04246BE383}" name="Technique Used" dataDxfId="53"/>
+    <tableColumn id="1" xr3:uid="{2744E4B1-F4AF-4C38-A165-A36AFDC6ED20}" name="Test Case ID" dataDxfId="116"/>
+    <tableColumn id="2" xr3:uid="{025A828A-E3BB-46BB-9738-33A224653725}" name="Test Suite" dataDxfId="115"/>
+    <tableColumn id="3" xr3:uid="{63419378-8000-4158-90E8-6D8BFCDA2241}" name="Test Title" dataDxfId="114"/>
+    <tableColumn id="4" xr3:uid="{485947B2-61B2-4E7A-9F45-DEE2A6A31241}" name="Preconditions" dataDxfId="113"/>
+    <tableColumn id="5" xr3:uid="{694A91C3-2EF7-4662-BA6E-D1E59F3B94D5}" name="Test Steps" dataDxfId="112"/>
+    <tableColumn id="6" xr3:uid="{61B98F31-1685-42B6-BF1B-14C77B125CFB}" name="Expected Result" dataDxfId="111"/>
+    <tableColumn id="7" xr3:uid="{C5850C5A-CF04-45AE-AFF2-FF9A3159C7A6}" name="Actual Result" dataDxfId="110"/>
+    <tableColumn id="8" xr3:uid="{880E8ECB-3308-49AD-B50B-5CCE1EF7E617}" name="Pass/Fail" dataDxfId="109"/>
+    <tableColumn id="9" xr3:uid="{4F749DFF-645B-47DB-9AAC-12B65CE23CB3}" name="Defect Reference" dataDxfId="108"/>
+    <tableColumn id="10" xr3:uid="{A573EAAC-61E8-4701-AA89-F5788D455FC0}" name="Priority" dataDxfId="107"/>
+    <tableColumn id="11" xr3:uid="{8507D1F9-0769-438C-86B4-E44A8C17EF24}" name="Test Type" dataDxfId="106"/>
+    <tableColumn id="12" xr3:uid="{ADF76C2E-E815-4CC9-B9BC-DE04246BE383}" name="Technique Used" dataDxfId="105"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B781F207-FC8D-435D-8A2A-008198199B42}" name="Table1345" displayName="Table1345" ref="A1:L35" totalsRowShown="0" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B781F207-FC8D-435D-8A2A-008198199B42}" name="Table1345" displayName="Table1345" ref="A1:L35" totalsRowShown="0" dataDxfId="143">
   <autoFilter ref="A1:L35" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{6EF8EB41-2551-44C0-81AD-6983683B3589}" name="Test Case ID" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{6FADDCBB-6A26-4047-BF85-6CC1B18AD9DE}" name="Test Suite" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{36BE9279-D322-4751-A8AE-1455D7F93425}" name="Test Title" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{AD6615BC-F350-4794-ABAE-EFC9B39D63F9}" name="Preconditions" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{E85963AF-AD48-4BC5-8B46-91ED9A9A5239}" name="Test Steps" dataDxfId="47"/>
-    <tableColumn id="6" xr3:uid="{B4E896D7-5A65-4028-BFA8-6BF5F0C80AB5}" name="Expected Result" dataDxfId="46"/>
-    <tableColumn id="7" xr3:uid="{B55753B6-0BAF-4862-8D03-9EFB37E556F3}" name="Actual Result" dataDxfId="45"/>
-    <tableColumn id="8" xr3:uid="{757CEF9C-9579-4CEB-A8BA-4C87F61F8686}" name="Pass/Fail" dataDxfId="44"/>
-    <tableColumn id="9" xr3:uid="{180213C5-DA7E-4959-88B0-CF50B9672E2F}" name="Defect Reference" dataDxfId="43"/>
-    <tableColumn id="10" xr3:uid="{B21A2342-3987-4CA6-A6AE-F1C3DF81993D}" name="Priority" dataDxfId="42"/>
-    <tableColumn id="11" xr3:uid="{17FBF0DF-5ED1-43F3-B1FC-D7191352E182}" name="Test Type" dataDxfId="41"/>
-    <tableColumn id="12" xr3:uid="{F08D4311-D55F-4CE9-88B2-87547B0D8598}" name="Technique Used" dataDxfId="40"/>
+    <tableColumn id="1" xr3:uid="{6EF8EB41-2551-44C0-81AD-6983683B3589}" name="Test Case ID" dataDxfId="142"/>
+    <tableColumn id="2" xr3:uid="{6FADDCBB-6A26-4047-BF85-6CC1B18AD9DE}" name="Test Suite" dataDxfId="141"/>
+    <tableColumn id="3" xr3:uid="{36BE9279-D322-4751-A8AE-1455D7F93425}" name="Test Title" dataDxfId="140"/>
+    <tableColumn id="4" xr3:uid="{AD6615BC-F350-4794-ABAE-EFC9B39D63F9}" name="Preconditions" dataDxfId="139"/>
+    <tableColumn id="5" xr3:uid="{E85963AF-AD48-4BC5-8B46-91ED9A9A5239}" name="Test Steps" dataDxfId="138"/>
+    <tableColumn id="6" xr3:uid="{B4E896D7-5A65-4028-BFA8-6BF5F0C80AB5}" name="Expected Result" dataDxfId="137"/>
+    <tableColumn id="7" xr3:uid="{B55753B6-0BAF-4862-8D03-9EFB37E556F3}" name="Actual Result" dataDxfId="136"/>
+    <tableColumn id="8" xr3:uid="{757CEF9C-9579-4CEB-A8BA-4C87F61F8686}" name="Pass/Fail" dataDxfId="135"/>
+    <tableColumn id="9" xr3:uid="{180213C5-DA7E-4959-88B0-CF50B9672E2F}" name="Defect Reference" dataDxfId="134"/>
+    <tableColumn id="10" xr3:uid="{B21A2342-3987-4CA6-A6AE-F1C3DF81993D}" name="Priority" dataDxfId="133"/>
+    <tableColumn id="11" xr3:uid="{17FBF0DF-5ED1-43F3-B1FC-D7191352E182}" name="Test Type" dataDxfId="132"/>
+    <tableColumn id="12" xr3:uid="{F08D4311-D55F-4CE9-88B2-87547B0D8598}" name="Technique Used" dataDxfId="131"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61AE62D4-A34D-4905-9EA9-E9E0F4B9116A}" name="Table134" displayName="Table134" ref="A1:L25" totalsRowShown="0" dataDxfId="39">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{61AE62D4-A34D-4905-9EA9-E9E0F4B9116A}" name="Table134" displayName="Table134" ref="A1:L25" totalsRowShown="0" dataDxfId="104">
   <autoFilter ref="A1:L25" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{612D3960-86E1-4810-993F-4862815DDA7E}" name="Test Case ID" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{48491056-2F89-4C99-B221-A154C135DD8B}" name="Test Suite" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{C379C391-DF6E-498E-9B62-0ABF6B6BBA4F}" name="Test Title" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{198C39E7-1666-44F1-BBF9-04456774642F}" name="Preconditions" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{73A8B408-432E-48DF-A1C3-CB4F67389659}" name="Test Steps" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{A9872DF8-F94C-4362-891B-9103348329E0}" name="Expected Result" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{F97A4672-76D0-4966-BE44-84EF3775F758}" name="Actual Result" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{F5AD4938-A73F-40DE-A458-F4C98DB74708}" name="Pass/Fail" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{4EB9106A-08E3-4179-AB0C-A24C70F775D2}" name="Defect Reference" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{533762C2-81B6-41A2-959B-5727C9A9EB9F}" name="Priority" dataDxfId="29"/>
-    <tableColumn id="11" xr3:uid="{8DB1E476-6483-4F65-BBA1-2E0315BAE2D7}" name="Test Type" dataDxfId="28"/>
-    <tableColumn id="12" xr3:uid="{A98AEC51-2FB9-43FA-9055-F78DD7613D88}" name="Technique Used" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{612D3960-86E1-4810-993F-4862815DDA7E}" name="Test Case ID" dataDxfId="103"/>
+    <tableColumn id="2" xr3:uid="{48491056-2F89-4C99-B221-A154C135DD8B}" name="Test Suite" dataDxfId="102"/>
+    <tableColumn id="3" xr3:uid="{C379C391-DF6E-498E-9B62-0ABF6B6BBA4F}" name="Test Title" dataDxfId="101"/>
+    <tableColumn id="4" xr3:uid="{198C39E7-1666-44F1-BBF9-04456774642F}" name="Preconditions" dataDxfId="100"/>
+    <tableColumn id="5" xr3:uid="{73A8B408-432E-48DF-A1C3-CB4F67389659}" name="Test Steps" dataDxfId="99"/>
+    <tableColumn id="6" xr3:uid="{A9872DF8-F94C-4362-891B-9103348329E0}" name="Expected Result" dataDxfId="98"/>
+    <tableColumn id="7" xr3:uid="{F97A4672-76D0-4966-BE44-84EF3775F758}" name="Actual Result" dataDxfId="97"/>
+    <tableColumn id="8" xr3:uid="{F5AD4938-A73F-40DE-A458-F4C98DB74708}" name="Pass/Fail" dataDxfId="96"/>
+    <tableColumn id="9" xr3:uid="{4EB9106A-08E3-4179-AB0C-A24C70F775D2}" name="Defect Reference" dataDxfId="95"/>
+    <tableColumn id="10" xr3:uid="{533762C2-81B6-41A2-959B-5727C9A9EB9F}" name="Priority" dataDxfId="94"/>
+    <tableColumn id="11" xr3:uid="{8DB1E476-6483-4F65-BBA1-2E0315BAE2D7}" name="Test Type" dataDxfId="93"/>
+    <tableColumn id="12" xr3:uid="{A98AEC51-2FB9-43FA-9055-F78DD7613D88}" name="Technique Used" dataDxfId="92"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0D196AD6-EF67-4A66-8E49-8C2841204709}" name="Table13456" displayName="Table13456" ref="A1:L12" totalsRowShown="0" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{0D196AD6-EF67-4A66-8E49-8C2841204709}" name="Table13456" displayName="Table13456" ref="A1:L12" totalsRowShown="0" dataDxfId="91">
   <autoFilter ref="A1:L12" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{466CEFD5-F045-49B3-AF42-A537C929F3BE}" name="Test Case ID" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{41E139CF-000A-4FEE-A5CF-7F36FD2168EA}" name="Test Suite" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{D8F34F80-4930-477A-ACDA-B2E1D2C03810}" name="Test Title" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{8ADBF18A-BE48-4A82-B8D1-B9D361A9D77F}" name="Preconditions" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{5FF95E03-9624-497C-A9AD-46F99B729C31}" name="Test Steps" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{0A77C29C-5E72-468E-9846-655DE8ADDD82}" name="Expected Result" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{4EDC0818-C3F5-469B-ABD0-1D2636966782}" name="Actual Result" dataDxfId="19"/>
-    <tableColumn id="8" xr3:uid="{A91EAE30-2BAD-42CE-B0AE-954D35FEA9CB}" name="Pass/Fail" dataDxfId="18"/>
-    <tableColumn id="9" xr3:uid="{5D452F4E-9031-4F8D-B186-1DAFF9582E38}" name="Defect Reference" dataDxfId="17"/>
-    <tableColumn id="10" xr3:uid="{E664542B-8BA2-4D22-9AEA-F6D9F8027E11}" name="Priority" dataDxfId="16"/>
-    <tableColumn id="11" xr3:uid="{F6021F5E-78C9-407E-BED7-F5E43381CF73}" name="Test Type" dataDxfId="15"/>
-    <tableColumn id="12" xr3:uid="{C9082BF6-5D7D-4CE4-B9F1-A9815761046D}" name="Technique Used" dataDxfId="14"/>
+    <tableColumn id="1" xr3:uid="{466CEFD5-F045-49B3-AF42-A537C929F3BE}" name="Test Case ID" dataDxfId="90"/>
+    <tableColumn id="2" xr3:uid="{41E139CF-000A-4FEE-A5CF-7F36FD2168EA}" name="Test Suite" dataDxfId="89"/>
+    <tableColumn id="3" xr3:uid="{D8F34F80-4930-477A-ACDA-B2E1D2C03810}" name="Test Title" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{8ADBF18A-BE48-4A82-B8D1-B9D361A9D77F}" name="Preconditions" dataDxfId="87"/>
+    <tableColumn id="5" xr3:uid="{5FF95E03-9624-497C-A9AD-46F99B729C31}" name="Test Steps" dataDxfId="86"/>
+    <tableColumn id="6" xr3:uid="{0A77C29C-5E72-468E-9846-655DE8ADDD82}" name="Expected Result" dataDxfId="85"/>
+    <tableColumn id="7" xr3:uid="{4EDC0818-C3F5-469B-ABD0-1D2636966782}" name="Actual Result" dataDxfId="84"/>
+    <tableColumn id="8" xr3:uid="{A91EAE30-2BAD-42CE-B0AE-954D35FEA9CB}" name="Pass/Fail" dataDxfId="83"/>
+    <tableColumn id="9" xr3:uid="{5D452F4E-9031-4F8D-B186-1DAFF9582E38}" name="Defect Reference" dataDxfId="82"/>
+    <tableColumn id="10" xr3:uid="{E664542B-8BA2-4D22-9AEA-F6D9F8027E11}" name="Priority" dataDxfId="81"/>
+    <tableColumn id="11" xr3:uid="{F6021F5E-78C9-407E-BED7-F5E43381CF73}" name="Test Type" dataDxfId="80"/>
+    <tableColumn id="12" xr3:uid="{C9082BF6-5D7D-4CE4-B9F1-A9815761046D}" name="Technique Used" dataDxfId="79"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{F9565653-BE23-4F65-BB04-193CD2FC32A3}" name="Table134567" displayName="Table134567" ref="A1:L22" totalsRowShown="0" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{F9565653-BE23-4F65-BB04-193CD2FC32A3}" name="Table134567" displayName="Table134567" ref="A1:L22" totalsRowShown="0" dataDxfId="78">
   <autoFilter ref="A1:L22" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{66C7640D-5314-4210-BD3C-8E45AFC1300F}" name="Test Case ID" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{4F21B4A4-0812-437C-8C07-D42183C50C61}" name="Test Suite" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{6262FB8E-2325-43FA-9936-1E7E03B1A6D9}" name="Test Title" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{BFCA6D0B-2C78-4AC8-91B5-F4DA2EE06B2B}" name="Preconditions" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{D1414F7A-E2A7-49A3-B3A7-FEE7B53CB384}" name="Test Steps" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{4D176B05-3EF0-44E8-A906-797ED16711E9}" name="Expected Result" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{C73A291E-BBB4-41C0-B256-E899F57AFAE5}" name="Actual Result" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{7826C864-39AB-46DC-AAB3-3EB73C32300C}" name="Pass/Fail" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{D417C83F-B82D-4910-B09B-2CB370C85443}" name="Defect Reference" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{87D08049-B3A1-43E8-9228-C261B30195CD}" name="Priority" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{B3BB6C34-4394-43A0-8A94-418EAC9CE420}" name="Test Type" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{0E657545-54E7-4F7E-8A52-9EA26C90EF6F}" name="Technique Used" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{66C7640D-5314-4210-BD3C-8E45AFC1300F}" name="Test Case ID" dataDxfId="77"/>
+    <tableColumn id="2" xr3:uid="{4F21B4A4-0812-437C-8C07-D42183C50C61}" name="Test Suite" dataDxfId="76"/>
+    <tableColumn id="3" xr3:uid="{6262FB8E-2325-43FA-9936-1E7E03B1A6D9}" name="Test Title" dataDxfId="75"/>
+    <tableColumn id="4" xr3:uid="{BFCA6D0B-2C78-4AC8-91B5-F4DA2EE06B2B}" name="Preconditions" dataDxfId="74"/>
+    <tableColumn id="5" xr3:uid="{D1414F7A-E2A7-49A3-B3A7-FEE7B53CB384}" name="Test Steps" dataDxfId="73"/>
+    <tableColumn id="6" xr3:uid="{4D176B05-3EF0-44E8-A906-797ED16711E9}" name="Expected Result" dataDxfId="72"/>
+    <tableColumn id="7" xr3:uid="{C73A291E-BBB4-41C0-B256-E899F57AFAE5}" name="Actual Result" dataDxfId="71"/>
+    <tableColumn id="8" xr3:uid="{7826C864-39AB-46DC-AAB3-3EB73C32300C}" name="Pass/Fail" dataDxfId="70"/>
+    <tableColumn id="9" xr3:uid="{D417C83F-B82D-4910-B09B-2CB370C85443}" name="Defect Reference" dataDxfId="69"/>
+    <tableColumn id="10" xr3:uid="{87D08049-B3A1-43E8-9228-C261B30195CD}" name="Priority" dataDxfId="68"/>
+    <tableColumn id="11" xr3:uid="{B3BB6C34-4394-43A0-8A94-418EAC9CE420}" name="Test Type" dataDxfId="67"/>
+    <tableColumn id="12" xr3:uid="{0E657545-54E7-4F7E-8A52-9EA26C90EF6F}" name="Technique Used" dataDxfId="66"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3D805676-EB36-400A-A75C-B3DB5F605C86}" name="Table1345678" displayName="Table1345678" ref="A1:L21" totalsRowShown="0" dataDxfId="91">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3D805676-EB36-400A-A75C-B3DB5F605C86}" name="Table1345678" displayName="Table1345678" ref="A1:L21" totalsRowShown="0" dataDxfId="65">
   <autoFilter ref="A1:L21" xr:uid="{FA35CE46-814C-46D1-9769-58FB69203646}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{D2AF045E-8B07-4980-81C0-317EA0A3458C}" name="Test Case ID" dataDxfId="90"/>
-    <tableColumn id="2" xr3:uid="{12EA3EC5-2C4A-4EC6-A6C0-09BCD39015EB}" name="Test Suite" dataDxfId="89"/>
-    <tableColumn id="3" xr3:uid="{CD6F3C75-172A-4A6D-AAF9-9767D46C511F}" name="Test Title" dataDxfId="88"/>
-    <tableColumn id="4" xr3:uid="{11C37EC2-6309-4F28-A4F6-3530F57F081D}" name="Preconditions" dataDxfId="87"/>
-    <tableColumn id="5" xr3:uid="{348BF535-E0E2-4928-A257-B51A00A86CA9}" name="Test Steps" dataDxfId="86"/>
-    <tableColumn id="6" xr3:uid="{87E6DBB7-E575-4DE0-8FE9-455DF49CC89F}" name="Expected Result" dataDxfId="85"/>
-    <tableColumn id="7" xr3:uid="{4B0E423D-97D5-4BC9-8865-E7381703ACDC}" name="Actual Result" dataDxfId="84"/>
-    <tableColumn id="8" xr3:uid="{7D1050FA-7F67-463D-B4E4-17BDAB0E7D31}" name="Pass/Fail" dataDxfId="83"/>
-    <tableColumn id="9" xr3:uid="{99EFD087-DFF5-4CEF-8CFA-DAA78720FAFB}" name="Defect Reference" dataDxfId="82"/>
-    <tableColumn id="10" xr3:uid="{238DBB85-657F-49C9-84B3-889041D18F19}" name="Priority" dataDxfId="81"/>
-    <tableColumn id="11" xr3:uid="{984D9A05-D95A-4B4B-9D9A-6F1126B14801}" name="Test Type" dataDxfId="80"/>
-    <tableColumn id="12" xr3:uid="{D9955BB5-281C-4985-905F-A21D3A2F195A}" name="Technique Used" dataDxfId="79"/>
+    <tableColumn id="1" xr3:uid="{D2AF045E-8B07-4980-81C0-317EA0A3458C}" name="Test Case ID" dataDxfId="64"/>
+    <tableColumn id="2" xr3:uid="{12EA3EC5-2C4A-4EC6-A6C0-09BCD39015EB}" name="Test Suite" dataDxfId="63"/>
+    <tableColumn id="3" xr3:uid="{CD6F3C75-172A-4A6D-AAF9-9767D46C511F}" name="Test Title" dataDxfId="62"/>
+    <tableColumn id="4" xr3:uid="{11C37EC2-6309-4F28-A4F6-3530F57F081D}" name="Preconditions" dataDxfId="61"/>
+    <tableColumn id="5" xr3:uid="{348BF535-E0E2-4928-A257-B51A00A86CA9}" name="Test Steps" dataDxfId="60"/>
+    <tableColumn id="6" xr3:uid="{87E6DBB7-E575-4DE0-8FE9-455DF49CC89F}" name="Expected Result" dataDxfId="59"/>
+    <tableColumn id="7" xr3:uid="{4B0E423D-97D5-4BC9-8865-E7381703ACDC}" name="Actual Result" dataDxfId="58"/>
+    <tableColumn id="8" xr3:uid="{7D1050FA-7F67-463D-B4E4-17BDAB0E7D31}" name="Pass/Fail" dataDxfId="57"/>
+    <tableColumn id="9" xr3:uid="{99EFD087-DFF5-4CEF-8CFA-DAA78720FAFB}" name="Defect Reference" dataDxfId="56"/>
+    <tableColumn id="10" xr3:uid="{238DBB85-657F-49C9-84B3-889041D18F19}" name="Priority" dataDxfId="55"/>
+    <tableColumn id="11" xr3:uid="{984D9A05-D95A-4B4B-9D9A-6F1126B14801}" name="Test Type" dataDxfId="54"/>
+    <tableColumn id="12" xr3:uid="{D9955BB5-281C-4985-905F-A21D3A2F195A}" name="Technique Used" dataDxfId="53"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DAC3046E-7A50-4FD7-8453-9FC8DC11B96D}" name="Table19" displayName="Table19" ref="A1:F9" totalsRowShown="0" headerRowDxfId="52" dataDxfId="45">
+  <autoFilter ref="A1:F9" xr:uid="{DAC3046E-7A50-4FD7-8453-9FC8DC11B96D}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{1A5CC2C1-1E62-4E00-864A-82A2FC930B38}" name="ID" dataDxfId="51"/>
+    <tableColumn id="2" xr3:uid="{D0E4F0DB-5792-4907-A45A-069E3B91B00F}" name="Rule 1: _x000a_Is Account Active?" dataDxfId="50"/>
+    <tableColumn id="3" xr3:uid="{A7A6E5E4-EBE4-4699-BEA3-4B22B45D34DF}" name="Rule 2:_x000a_Does Account Have Sufficient Funds?" dataDxfId="49"/>
+    <tableColumn id="4" xr3:uid="{E61A47B0-F5DB-4CEF-8768-78CCF259235F}" name="Rule 3:_x000a_Under Daily Limit?" dataDxfId="48"/>
+    <tableColumn id="5" xr3:uid="{E2B16109-A64E-41E4-B5C9-D48E58E84521}" name="Expected Outcome" dataDxfId="47"/>
+    <tableColumn id="6" xr3:uid="{C385D04B-D65F-413D-A449-D58B14ECBBE7}" name="Expected Error Message If Not True" dataDxfId="46"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="18" xr:uid="{23FA6A11-A35C-4F11-857D-88C08503F56A}" name="Table12" displayName="Table12" ref="A2:E11" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="A2:E11" xr:uid="{23FA6A11-A35C-4F11-857D-88C08503F56A}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{60B4BB32-1420-4B69-9F19-0AF13A1E2F45}" name="Test Case ID" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{E7FD3624-D6D9-4FAA-9E28-68C73BD4E7DD}" name="Current State" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{CB809305-1896-479C-BECD-17AEFC49CDA6}" name="Transition Trigger" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{E802CF9E-B675-43F2-92DB-10381D5FA3B1}" name="Expected State" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{7CC69119-A773-4E68-9DC2-892539A1F0B6}" name="Actual State" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4439,7 +5609,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="O2">
-    <cfRule type="cellIs" dxfId="0" priority="15" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="15" operator="greaterThan">
       <formula>#REF!</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4447,6 +5617,621 @@
   <pageSetup scale="35" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
     <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E76AE919-0A35-45DB-8C8F-40136F6039FB}">
+  <sheetPr>
+    <tabColor theme="9"/>
+  </sheetPr>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="40.85546875" customWidth="1"/>
+    <col min="2" max="2" width="44.85546875" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="24.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>918</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>919</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>920</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>921</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>922</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>923</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>924</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>925</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>926</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>927</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>928</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>929</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>930</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>931</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>932</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>933</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>934</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>960</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>935</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>936</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>937</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>938</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>939</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>940</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>941</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>942</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>943</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>944</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>945</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>946</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>947</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>948</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>949</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>964</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>950</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>951</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>952</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>953</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>954</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>955</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>956</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60606D4E-4E9A-4F3A-9493-C0D30717EAF2}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.7109375" customWidth="1"/>
+    <col min="2" max="2" width="44.5703125" customWidth="1"/>
+    <col min="3" max="3" width="37.5703125" customWidth="1"/>
+    <col min="4" max="4" width="30.28515625" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" customWidth="1"/>
+    <col min="6" max="6" width="35.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>780</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+    </row>
+    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>781</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>782</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>783</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>785</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>786</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>787</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>788</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F3" s="9"/>
+    </row>
+    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="9" t="s">
+        <v>789</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>790</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>791</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>792</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F4" s="9"/>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="9" t="s">
+        <v>793</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>794</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>795</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>796</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F5" s="9"/>
+    </row>
+    <row r="6" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A6" s="9" t="s">
+        <v>797</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>798</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>799</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>800</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F6" s="9"/>
+    </row>
+    <row r="7" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>801</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>802</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>803</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>804</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>805</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>806</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>807</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>808</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F8" s="9"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>809</v>
+      </c>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>810</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>811</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>812</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="1"/>
+    </row>
+    <row r="11" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>813</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>814</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>815</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>816</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
+        <v>817</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>818</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>819</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>820</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
+        <v>821</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>822</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>823</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>824</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>825</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>826</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>827</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>828</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F14" s="1"/>
+    </row>
+    <row r="15" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>829</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>830</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>831</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>832</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>567</v>
+      </c>
+      <c r="F15" s="1"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>833</v>
+      </c>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>834</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>835</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>836</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>837</v>
+      </c>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>838</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>839</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>840</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>698</v>
+      </c>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>842</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>844</v>
+      </c>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+    </row>
+    <row r="20" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>845</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>846</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>847</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>848</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>849</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>850</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>851</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>852</v>
+      </c>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+    </row>
+    <row r="22" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>853</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>854</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>856</v>
+      </c>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+    </row>
+    <row r="23" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>857</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>858</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>859</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>860</v>
+      </c>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A9:E9"/>
+    <mergeCell ref="A16:E16"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="3">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -10074,4 +11859,611 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ACE8E78-2D2F-4A0B-9070-31EFFA5F5861}">
+  <sheetPr>
+    <tabColor theme="9"/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="32.7109375" customWidth="1"/>
+    <col min="2" max="2" width="22.140625" customWidth="1"/>
+    <col min="3" max="3" width="31.42578125" customWidth="1"/>
+    <col min="4" max="4" width="29.85546875" customWidth="1"/>
+    <col min="5" max="5" width="24.5703125" customWidth="1"/>
+    <col min="6" max="6" width="39.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="90" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>758</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>759</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>760</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>762</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>764</v>
+      </c>
+      <c r="B2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="D2" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>766</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="B3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="D3" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>771</v>
+      </c>
+      <c r="B4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>773</v>
+      </c>
+      <c r="B5" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="D5" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>775</v>
+      </c>
+      <c r="B6" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>776</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="C7" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>765</v>
+      </c>
+      <c r="D8" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>779</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>777</v>
+      </c>
+      <c r="C9" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>769</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>770</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{247F76D8-9589-4EE4-8D4A-0FB4FF5EA98F}">
+  <sheetPr>
+    <tabColor theme="8"/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.85546875" customWidth="1"/>
+    <col min="3" max="4" width="27.7109375" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
+        <v>861</v>
+      </c>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>862</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>863</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>864</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>866</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>868</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>870</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>871</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>872</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>872</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>873</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>872</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>874</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>875</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>872</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>876</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>877</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>878</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>876</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>877</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>877</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>879</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>877</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>880</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>882</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>884</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>885</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>886</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>887</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>888</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>889</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>887</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>890</v>
+      </c>
+      <c r="B12" s="11"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+    </row>
+    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>862</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>863</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>864</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>891</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>892</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>896</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>896</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>893</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>896</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>917</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>895</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>894</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>914</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>897</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>900</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>869</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>904</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>869</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>902</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>903</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>907</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>905</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>906</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>909</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>908</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>906</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>911</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>910</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>906</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>916</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>896</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>912</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>906</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>906</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A12:E12"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>